<commit_message>
Por filial - PRONTO
</commit_message>
<xml_diff>
--- a/Documentos/ManutRolo.xlsx
+++ b/Documentos/ManutRolo.xlsx
@@ -10,7 +10,7 @@
     <sheet sheetId="1" r:id="rId1" name="ManutRolo"/>
   </sheets>
   <definedNames>
-    <definedName name="ManutRolo">'ManutRolo'!$A$1:$K$1392</definedName>
+    <definedName name="ManutRolo">'ManutRolo'!$A$1:$K$1405</definedName>
   </definedNames>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
@@ -347,7 +347,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1392"/>
+  <dimension ref="A1:K1405"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row outlineLevel="0" r="1">
@@ -60182,7 +60182,7 @@
         <v>1394</v>
       </c>
       <c r="B1392" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C1392" s="0">
         <v>2</v>
@@ -60192,15 +60192,15 @@
       </c>
       <c r="E1392" s="0" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>ROLOTIPO</t>
         </is>
       </c>
       <c r="F1392" s="1">
-        <v>45611</v>
+        <v>45645</v>
       </c>
       <c r="G1392" s="0" t="inlineStr">
         <is>
-          <t>DSFJSDLFJSDFJLKSDJFKLSDJFKLSDVKLSVKSDVNSDVL</t>
+          <t>BORRACHA INCHADA.</t>
         </is>
       </c>
       <c r="H1392" s="0" t="inlineStr">
@@ -60209,15 +60209,574 @@
         </is>
       </c>
       <c r="I1392" s="1">
-        <v>45623.3536111111</v>
+        <v>45646.5725115741</v>
       </c>
       <c r="J1392" s="0" t="inlineStr">
         <is>
-          <t>gffernandes</t>
+          <t>rduarte</t>
         </is>
       </c>
       <c r="K1392" s="0">
-        <v>15000</v>
+        <v>262729</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1393">
+      <c r="A1393" s="0">
+        <v>1395</v>
+      </c>
+      <c r="B1393" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1393" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1393" s="0">
+        <v>7</v>
+      </c>
+      <c r="E1393" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1393" s="1">
+        <v>45645</v>
+      </c>
+      <c r="G1393" s="0" t="inlineStr">
+        <is>
+          <t>SUBSTITUIR ROLAMENTO.</t>
+        </is>
+      </c>
+      <c r="H1393" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1393" s="1">
+        <v>45646.5734027778</v>
+      </c>
+      <c r="J1393" s="0" t="inlineStr">
+        <is>
+          <t>rduarte</t>
+        </is>
+      </c>
+      <c r="K1393" s="0">
+        <v>262729</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1394">
+      <c r="A1394" s="0">
+        <v>1396</v>
+      </c>
+      <c r="B1394" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1394" s="0">
+        <v>2</v>
+      </c>
+      <c r="D1394" s="0">
+        <v>8</v>
+      </c>
+      <c r="E1394" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1394" s="1">
+        <v>45645</v>
+      </c>
+      <c r="G1394" s="0" t="inlineStr">
+        <is>
+          <t>BORRACHA INCHADA.</t>
+        </is>
+      </c>
+      <c r="H1394" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1394" s="1">
+        <v>45646.5740277778</v>
+      </c>
+      <c r="J1394" s="0" t="inlineStr">
+        <is>
+          <t>rduarte</t>
+        </is>
+      </c>
+      <c r="K1394" s="0">
+        <v>262729</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1395">
+      <c r="A1395" s="0">
+        <v>1397</v>
+      </c>
+      <c r="B1395" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1395" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1395" s="0">
+        <v>1</v>
+      </c>
+      <c r="E1395" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1395" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1395" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1395" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1395" s="1">
+        <v>45722.4051273148</v>
+      </c>
+      <c r="J1395" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1395" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1396">
+      <c r="A1396" s="0">
+        <v>1398</v>
+      </c>
+      <c r="B1396" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1396" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1396" s="0">
+        <v>5</v>
+      </c>
+      <c r="E1396" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1396" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1396" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1396" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1396" s="1">
+        <v>45722.405775463</v>
+      </c>
+      <c r="J1396" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1396" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1397">
+      <c r="A1397" s="0">
+        <v>1399</v>
+      </c>
+      <c r="B1397" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1397" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1397" s="0">
+        <v>6</v>
+      </c>
+      <c r="E1397" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1397" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1397" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1397" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1397" s="1">
+        <v>45722.4063425926</v>
+      </c>
+      <c r="J1397" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1397" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1398">
+      <c r="A1398" s="0">
+        <v>1400</v>
+      </c>
+      <c r="B1398" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1398" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1398" s="0">
+        <v>7</v>
+      </c>
+      <c r="E1398" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1398" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1398" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1398" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1398" s="1">
+        <v>45722.4067939815</v>
+      </c>
+      <c r="J1398" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1398" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1399">
+      <c r="A1399" s="0">
+        <v>1401</v>
+      </c>
+      <c r="B1399" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1399" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1399" s="0">
+        <v>8</v>
+      </c>
+      <c r="E1399" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1399" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1399" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1399" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1399" s="1">
+        <v>45722.4071875</v>
+      </c>
+      <c r="J1399" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1399" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1400">
+      <c r="A1400" s="0">
+        <v>1402</v>
+      </c>
+      <c r="B1400" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1400" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1400" s="0">
+        <v>9</v>
+      </c>
+      <c r="E1400" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1400" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1400" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1400" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1400" s="1">
+        <v>45722.4076967593</v>
+      </c>
+      <c r="J1400" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1400" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1401">
+      <c r="A1401" s="0">
+        <v>1403</v>
+      </c>
+      <c r="B1401" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1401" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1401" s="0">
+        <v>10</v>
+      </c>
+      <c r="E1401" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1401" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1401" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1401" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1401" s="1">
+        <v>45722.4080671296</v>
+      </c>
+      <c r="J1401" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1401" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1402">
+      <c r="A1402" s="0">
+        <v>1404</v>
+      </c>
+      <c r="B1402" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1402" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1402" s="0">
+        <v>11</v>
+      </c>
+      <c r="E1402" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1402" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1402" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1402" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1402" s="1">
+        <v>45722.4084375</v>
+      </c>
+      <c r="J1402" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1402" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1403">
+      <c r="A1403" s="0">
+        <v>1405</v>
+      </c>
+      <c r="B1403" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1403" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1403" s="0">
+        <v>12</v>
+      </c>
+      <c r="E1403" s="0" t="inlineStr">
+        <is>
+          <t>--------</t>
+        </is>
+      </c>
+      <c r="F1403" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1403" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA - SUBSTITUIDO ROLAMENTOS</t>
+        </is>
+      </c>
+      <c r="H1403" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1403" s="1">
+        <v>45722.4088657407</v>
+      </c>
+      <c r="J1403" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1403" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1404">
+      <c r="A1404" s="0">
+        <v>1406</v>
+      </c>
+      <c r="B1404" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1404" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1404" s="0">
+        <v>14</v>
+      </c>
+      <c r="E1404" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1404" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1404" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1404" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1404" s="1">
+        <v>45722.4094097222</v>
+      </c>
+      <c r="J1404" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1404" s="0">
+        <v>266241</v>
+      </c>
+    </row>
+    <row outlineLevel="0" r="1405">
+      <c r="A1405" s="0">
+        <v>1407</v>
+      </c>
+      <c r="B1405" s="0">
+        <v>2</v>
+      </c>
+      <c r="C1405" s="0">
+        <v>5</v>
+      </c>
+      <c r="D1405" s="0">
+        <v>15</v>
+      </c>
+      <c r="E1405" s="0" t="inlineStr">
+        <is>
+          <t>ROLOTIPO</t>
+        </is>
+      </c>
+      <c r="F1405" s="1">
+        <v>45714</v>
+      </c>
+      <c r="G1405" s="0" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="H1405" s="0" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="I1405" s="1">
+        <v>45722.4100462963</v>
+      </c>
+      <c r="J1405" s="0" t="inlineStr">
+        <is>
+          <t>lsouza</t>
+        </is>
+      </c>
+      <c r="K1405" s="0">
+        <v>266241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>